<commit_message>
feat(sigcom, ClosedAttention): modernize dashboard, implement cost type filter, columns highlighting, composed charts and compile updated data
</commit_message>
<xml_diff>
--- a/src/data/SIGCOM/SIGCOM 2026/(3) Marzo/Cubo 9_2026_03_121121_Hospital de Villarrica.xlsx
+++ b/src/data/SIGCOM/SIGCOM 2026/(3) Marzo/Cubo 9_2026_03_121121_Hospital de Villarrica.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vllhcontrol18\Escritorio\SIGCOM 2026\(3) Marzo\Nuevos formatos para enviar al minsal\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/22f23dde8628eee5/Aplicaciones Antigravity/Control de Gestion Web/src/data/SIGCOM/SIGCOM 2026/(3) Marzo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C17685E7-8310-418F-BC59-43C2360B20CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{C17685E7-8310-418F-BC59-43C2360B20CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{576E6A15-5D79-4CD8-A3E9-C536DC0D5929}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BEE5726E-9ECD-45CB-B94F-3448ED566828}"/>
   </bookViews>
@@ -578,10 +578,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="#,###"/>
-    <numFmt numFmtId="165" formatCode="#,##0_ ;\-#,##0\ "/>
-    <numFmt numFmtId="166" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="#,###"/>
+    <numFmt numFmtId="166" formatCode="#,##0_ ;\-#,##0\ "/>
+    <numFmt numFmtId="167" formatCode="yyyy/mm/dd"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -682,7 +682,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="20">
@@ -690,53 +690,53 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
@@ -775,9 +775,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -815,7 +815,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -921,7 +921,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1063,7 +1063,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -32355,9 +32355,7 @@
       <c r="C112" s="14">
         <v>0</v>
       </c>
-      <c r="D112" s="14">
-        <v>0</v>
-      </c>
+      <c r="D112" s="14"/>
       <c r="E112" s="14">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
fix(acuerdo, sigcom): mejorar espaciado lateral, remover selector redundante de servicio, agregar rango y-axis dinámico para metas y sincronizar datos SIGCOM de abril
</commit_message>
<xml_diff>
--- a/src/data/SIGCOM/SIGCOM 2026/(3) Marzo/Cubo 9_2026_03_121121_Hospital de Villarrica.xlsx
+++ b/src/data/SIGCOM/SIGCOM 2026/(3) Marzo/Cubo 9_2026_03_121121_Hospital de Villarrica.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/22f23dde8628eee5/Aplicaciones Antigravity/Control de Gestion Web/src/data/SIGCOM/SIGCOM 2026/(3) Marzo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Unidades compartidas\ASUR\SIGCOM\SIGCOM 2026\(3) Marzo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{C17685E7-8310-418F-BC59-43C2360B20CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{576E6A15-5D79-4CD8-A3E9-C536DC0D5929}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BABE0C6F-F0C2-4F28-8C7D-8D03AAA35A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BEE5726E-9ECD-45CB-B94F-3448ED566828}"/>
   </bookViews>
   <sheets>
     <sheet name="Cubo 9" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -583,7 +583,7 @@
     <numFmt numFmtId="166" formatCode="#,##0_ ;\-#,##0\ "/>
     <numFmt numFmtId="167" formatCode="yyyy/mm/dd"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -641,8 +641,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -653,6 +660,11 @@
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -680,12 +692,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -742,8 +755,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
+    <cellStyle name="Bueno" xfId="3" builtinId="26"/>
     <cellStyle name="Millares [0]" xfId="1" builtinId="6"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{B70C6238-5E80-4FCB-9083-4DC1A463EF60}"/>
@@ -1653,7 +1670,7 @@
       </c>
     </row>
     <row r="4" spans="2:96" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="20" t="s">
         <v>94</v>
       </c>
       <c r="C4" s="12">
@@ -4523,7 +4540,7 @@
       </c>
     </row>
     <row r="14" spans="2:96" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="20" t="s">
         <v>104</v>
       </c>
       <c r="C14" s="12">
@@ -15429,7 +15446,7 @@
       </c>
     </row>
     <row r="52" spans="2:96" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="11" t="s">
+      <c r="B52" s="20" t="s">
         <v>142</v>
       </c>
       <c r="C52" s="12">
@@ -32355,7 +32372,9 @@
       <c r="C112" s="14">
         <v>0</v>
       </c>
-      <c r="D112" s="14"/>
+      <c r="D112" s="14">
+        <v>0</v>
+      </c>
       <c r="E112" s="14">
         <v>0</v>
       </c>

</xml_diff>